<commit_message>
chore: retain institution name in attendance seed file while keeping employee names anonymized
</commit_message>
<xml_diff>
--- a/database/seeders/files/Absen 08 s.d 09 Jun.xlsx
+++ b/database/seeders/files/Absen 08 s.d 09 Jun.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1143">
   <si>
-    <t>RUMAH SAKIT UMUM DEMO</t>
+    <t>RS  BINTANG AMIN</t>
   </si>
   <si>
     <t>Total Time Card Report</t>
@@ -28,7 +28,7 @@
     <t>From  June 08 2026  To  June 09 2026</t>
   </si>
   <si>
-    <t>Company: RUMAH SAKIT UMUM DEMO</t>
+    <t>Company: RS  BINTANG AMIN</t>
   </si>
   <si>
     <t>Employee ID</t>

</xml_diff>